<commit_message>
feat: India Map, multi-doc per outlet, OCR cleanup, bill/supplementary extraction
- India Map on dashboard with react-simple-maps, 60+ city coordinates, hover tooltip cards
- Drive-like document management per outlet (upload/download/delete via Supabase storage)
- clean_ocr_text() post-processor for broken lines, whitespace, headers, OCR artifacts
- BILL_EXTRACTION_SCHEMA and SUPPLEMENTARY_AGREEMENT_SCHEMA for 5 document types
- Updated classify_document and extract_structured_data for bill + supplementary_agreement
- Updated Aryan task sheet with Batch 6 client feedback items
</commit_message>
<xml_diff>
--- a/GroSpace_Production_TaskSheet_Aryan.xlsx
+++ b/GroSpace_Production_TaskSheet_Aryan.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="29">
+  <fonts count="33">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -181,8 +181,27 @@
       <color rgb="004338CA"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00065F46"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00B45309"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -237,6 +256,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DCFCE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1FAE5"/>
       </patternFill>
     </fill>
   </fills>
@@ -310,7 +334,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -469,6 +493,18 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -835,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2261,14 +2297,6 @@
           <t>BATCH 5 — GOOGLE CLOUD VISION + ENHANCED Q&amp;A (NEW)</t>
         </is>
       </c>
-      <c r="B39" s="47" t="n"/>
-      <c r="C39" s="47" t="n"/>
-      <c r="D39" s="47" t="n"/>
-      <c r="E39" s="47" t="n"/>
-      <c r="F39" s="47" t="n"/>
-      <c r="G39" s="47" t="n"/>
-      <c r="H39" s="47" t="n"/>
-      <c r="I39" s="47" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="48" t="n">
@@ -2563,6 +2591,7 @@
         </is>
       </c>
     </row>
+    <row r="47"/>
     <row r="48">
       <c r="F48" s="54" t="inlineStr">
         <is>
@@ -2570,15 +2599,355 @@
         </is>
       </c>
       <c r="G48" s="54">
-        <f>SUM(G5:G46)</f>
+        <f>SUM(G5:G57)</f>
         <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="58" t="inlineStr">
+        <is>
+          <t>BATCH 6 — CLIENT FEEDBACK (India Map, Multi-Doc, OCR, Doc Types)</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n"/>
+      <c r="C49" s="5" t="n"/>
+      <c r="D49" s="5" t="n"/>
+      <c r="E49" s="5" t="n"/>
+      <c r="F49" s="5" t="n"/>
+      <c r="G49" s="5" t="n"/>
+      <c r="H49" s="5" t="n"/>
+      <c r="I49" s="6" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="59" t="n">
+        <v>38</v>
+      </c>
+      <c r="B50" s="59" t="inlineStr">
+        <is>
+          <t>Week 6</t>
+        </is>
+      </c>
+      <c r="C50" s="59" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="D50" s="59" t="inlineStr">
+        <is>
+          <t>India Map view on Dashboard</t>
+        </is>
+      </c>
+      <c r="E50" s="59" t="inlineStr">
+        <is>
+          <t>Add interactive India Map with react-simple-maps showing outlet locations by city. Hover tooltip cards show outlet name, status, rent. City sidebar with counts. Dynamic import with SSR disabled.</t>
+        </is>
+      </c>
+      <c r="F50" s="59" t="inlineStr">
+        <is>
+          <t>P1 HIGH</t>
+        </is>
+      </c>
+      <c r="G50" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="H50" s="60" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I50" s="59" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="59" t="n">
+        <v>39</v>
+      </c>
+      <c r="B51" s="59" t="inlineStr">
+        <is>
+          <t>Week 6</t>
+        </is>
+      </c>
+      <c r="C51" s="59" t="inlineStr">
+        <is>
+          <t>Frontend / Backend</t>
+        </is>
+      </c>
+      <c r="D51" s="59" t="inlineStr">
+        <is>
+          <t>Multiple documents per outlet (Drive-like)</t>
+        </is>
+      </c>
+      <c r="E51" s="59" t="inlineStr">
+        <is>
+          <t>Drive-like document management on outlet detail page. Upload/download/delete docs per outlet. Backend endpoints: GET/POST /api/outlets/{id}/documents, DELETE /api/documents/{id}. Supabase storage integration.</t>
+        </is>
+      </c>
+      <c r="F51" s="59" t="inlineStr">
+        <is>
+          <t>P1 HIGH</t>
+        </is>
+      </c>
+      <c r="G51" s="59" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H51" s="60" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I51" s="59" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="59" t="n">
+        <v>40</v>
+      </c>
+      <c r="B52" s="59" t="inlineStr">
+        <is>
+          <t>Week 6</t>
+        </is>
+      </c>
+      <c r="C52" s="59" t="inlineStr">
+        <is>
+          <t>Backend / AI</t>
+        </is>
+      </c>
+      <c r="D52" s="59" t="inlineStr">
+        <is>
+          <t>OCR text formatting &amp; cleanup</t>
+        </is>
+      </c>
+      <c r="E52" s="59" t="inlineStr">
+        <is>
+          <t>Add clean_ocr_text() post-processing function. Fixes broken lines, collapsed whitespace, removes page headers/footers, preserves table alignment, fixes common OCR character misreads. Applied to all text extraction paths.</t>
+        </is>
+      </c>
+      <c r="F52" s="59" t="inlineStr">
+        <is>
+          <t>P1 HIGH</t>
+        </is>
+      </c>
+      <c r="G52" s="59" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H52" s="60" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I52" s="59" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="59" t="n">
+        <v>41</v>
+      </c>
+      <c r="B53" s="59" t="inlineStr">
+        <is>
+          <t>Week 6</t>
+        </is>
+      </c>
+      <c r="C53" s="59" t="inlineStr">
+        <is>
+          <t>Backend / AI</t>
+        </is>
+      </c>
+      <c r="D53" s="59" t="inlineStr">
+        <is>
+          <t>Multiple document type extraction (Bill, Supplementary Agreement)</t>
+        </is>
+      </c>
+      <c r="E53" s="59" t="inlineStr">
+        <is>
+          <t>Add BILL_EXTRACTION_SCHEMA (electricity/water/tax/invoice) and SUPPLEMENTARY_AGREEMENT_SCHEMA (amendment/addendum). Update classify_document and extract_structured_data to handle 5 doc types: lease_loi, license_certificate, franchise_agreement, bill, supplementary_agreement.</t>
+        </is>
+      </c>
+      <c r="F53" s="59" t="inlineStr">
+        <is>
+          <t>P1 HIGH</t>
+        </is>
+      </c>
+      <c r="G53" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="H53" s="60" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I53" s="59" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="59" t="n">
+        <v>42</v>
+      </c>
+      <c r="B54" s="59" t="inlineStr">
+        <is>
+          <t>Week 6</t>
+        </is>
+      </c>
+      <c r="C54" s="59" t="inlineStr">
+        <is>
+          <t>Backend / Frontend</t>
+        </is>
+      </c>
+      <c r="D54" s="59" t="inlineStr">
+        <is>
+          <t>Role-based platform access — SLA tiered logins</t>
+        </is>
+      </c>
+      <c r="E54" s="59" t="inlineStr">
+        <is>
+          <t>Implement role tiers: CEO, CFO, Admin, Manager. Each role sees different dashboard widgets, has different permissions. CEO/CFO see portfolio-level metrics, Managers see outlet-level only. Enforce in both backend middleware and frontend route guards.</t>
+        </is>
+      </c>
+      <c r="F54" s="59" t="inlineStr">
+        <is>
+          <t>P1 HIGH</t>
+        </is>
+      </c>
+      <c r="G54" s="59" t="n">
+        <v>3</v>
+      </c>
+      <c r="H54" s="61" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I54" s="59" t="inlineStr">
+        <is>
+          <t>Extends existing role system (platform_admin, org_admin, org_member)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="59" t="n">
+        <v>43</v>
+      </c>
+      <c r="B55" s="59" t="inlineStr">
+        <is>
+          <t>Week 6</t>
+        </is>
+      </c>
+      <c r="C55" s="59" t="inlineStr">
+        <is>
+          <t>Backend / AI</t>
+        </is>
+      </c>
+      <c r="D55" s="59" t="inlineStr">
+        <is>
+          <t>Processing time estimates</t>
+        </is>
+      </c>
+      <c r="E55" s="59" t="inlineStr">
+        <is>
+          <t>Show estimated processing time before/during document upload. Track actual processing duration per doc type. Display progress bar with stage indicators (OCR → Classify → Extract → Risk Check).</t>
+        </is>
+      </c>
+      <c r="F55" s="59" t="inlineStr">
+        <is>
+          <t>P2 MEDIUM</t>
+        </is>
+      </c>
+      <c r="G55" s="59" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H55" s="61" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I55" s="59" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="59" t="n">
+        <v>44</v>
+      </c>
+      <c r="B56" s="59" t="inlineStr">
+        <is>
+          <t>Week 6</t>
+        </is>
+      </c>
+      <c r="C56" s="59" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="D56" s="59" t="inlineStr">
+        <is>
+          <t>Leasecake-style extraction UX</t>
+        </is>
+      </c>
+      <c r="E56" s="59" t="inlineStr">
+        <is>
+          <t>Model document extraction review on Leasecake UX patterns: inline field editing, section-by-section review, confidence badges per field, side-by-side PDF viewer with field highlighting.</t>
+        </is>
+      </c>
+      <c r="F56" s="59" t="inlineStr">
+        <is>
+          <t>P1 HIGH</t>
+        </is>
+      </c>
+      <c r="G56" s="59" t="n">
+        <v>2</v>
+      </c>
+      <c r="H56" s="61" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I56" s="59" t="inlineStr">
+        <is>
+          <t>Reference: Leasecake.com extraction flow</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="59" t="n">
+        <v>45</v>
+      </c>
+      <c r="B57" s="59" t="inlineStr">
+        <is>
+          <t>Week 6</t>
+        </is>
+      </c>
+      <c r="C57" s="59" t="inlineStr">
+        <is>
+          <t>Backend / Frontend</t>
+        </is>
+      </c>
+      <c r="D57" s="59" t="inlineStr">
+        <is>
+          <t>Google Sheet feedback pipeline</t>
+        </is>
+      </c>
+      <c r="E57" s="59" t="inlineStr">
+        <is>
+          <t>Create feedback mechanism: users can flag extraction errors or suggest corrections. Store feedback in a dedicated table. Auto-sync flagged items to a Google Sheet (via Google Sheets API) for team review.</t>
+        </is>
+      </c>
+      <c r="F57" s="59" t="inlineStr">
+        <is>
+          <t>P2 MEDIUM</t>
+        </is>
+      </c>
+      <c r="G57" s="59" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H57" s="61" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I57" s="59" t="inlineStr">
+        <is>
+          <t>Needs Google Sheets API credentials</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:I38"/>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A15:I15"/>
     <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A49:I49"/>
     <mergeCell ref="A5:I5"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A23:I23"/>
@@ -3459,7 +3828,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -4290,6 +4659,50 @@
       <c r="E44" s="57" t="inlineStr">
         <is>
           <t>NEW — Batch 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="62" t="inlineStr">
+        <is>
+          <t>GOOGLE_SHEETS_API_KEY</t>
+        </is>
+      </c>
+      <c r="B46" s="62" t="inlineStr">
+        <is>
+          <t>your-google-sheets-api-key</t>
+        </is>
+      </c>
+      <c r="C46" s="63" t="inlineStr">
+        <is>
+          <t>NEW — Week 6</t>
+        </is>
+      </c>
+      <c r="D46" s="62" t="inlineStr">
+        <is>
+          <t>Google Cloud Console → APIs → Credentials → Create API Key → Restrict to Sheets API</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="62" t="inlineStr">
+        <is>
+          <t>GOOGLE_SHEETS_SPREADSHEET_ID</t>
+        </is>
+      </c>
+      <c r="B47" s="62" t="inlineStr">
+        <is>
+          <t>1BxiMVs0XRA5nFMd...spreadsheet-id</t>
+        </is>
+      </c>
+      <c r="C47" s="63" t="inlineStr">
+        <is>
+          <t>NEW — Week 6</t>
+        </is>
+      </c>
+      <c r="D47" s="62" t="inlineStr">
+        <is>
+          <t>Create a Google Sheet for feedback → URL contains the spreadsheet ID</t>
         </is>
       </c>
     </row>

</xml_diff>